<commit_message>
total confusion matrix 수정
</commit_message>
<xml_diff>
--- a/연구코드/results/feature_selection/feature_selection_summary.xlsx
+++ b/연구코드/results/feature_selection/feature_selection_summary.xlsx
@@ -47,7 +47,7 @@
     <t>VIF pruning (VIF&gt;10)</t>
   </si>
   <si>
-    <t>slope_abs_mean, band4_energy, max, p25, fft_mag_std, band1_energy, median, p75, p10, wavelet_cA_energy, fft_mag_mean, p95, wavelet_cA_std, p90, peak_mean_height, AUC_normalized, mean_abs_deviation, spectral_rolloff, p5, wavelet_energy_ratio_D1, wavelet_cD2_energy, wavelet_cD1_energy, RMSE</t>
+    <t>max, fft_mag_std, wavelet_cA_std, p90, p5, p95, band1_energy, RMSE, p75, fft_mag_mean, band4_energy, wavelet_cD2_energy, peak_mean_height, slope_abs_mean, wavelet_cD1_energy, wavelet_energy_ratio_D1, p25, p10, AUC_normalized, median, wavelet_cA_energy, mean_abs_deviation, spectral_rolloff</t>
   </si>
   <si>
     <t>band1_energy_ratio, band3_energy_ratio, fft_mag_max, mean, p90_p10_ratio, peak_count, peak_last_pos, peak_main_pos, peak_max_height, peak_std_height, signal_length, slope_mean, slope_min, spectral_centroid, spectral_energy, valley_count, wavelet_cD1_std, wavelet_cD3_std, zero_crossing_rate</t>
@@ -83,15 +83,15 @@
     <t>vote_ge3</t>
   </si>
   <si>
+    <t>RF_Perm_only</t>
+  </si>
+  <si>
+    <t>vote_ge1</t>
+  </si>
+  <si>
     <t>union_all</t>
   </si>
   <si>
-    <t>vote_ge1</t>
-  </si>
-  <si>
-    <t>RF_Perm_only</t>
-  </si>
-  <si>
     <t>AUC, CV, IQR, band1_energy_ratio, band2_energy_ratio, kurtosis, p90_p10_ratio, peak_main_pos, peak_max_height, signal_energy, slope_mean, slope_min, zero_crossing_rate</t>
   </si>
   <si>
@@ -131,118 +131,118 @@
     <t>p_value</t>
   </si>
   <si>
+    <t>band1_energy_ratio</t>
+  </si>
+  <si>
+    <t>AUC</t>
+  </si>
+  <si>
     <t>slope_mean</t>
   </si>
   <si>
-    <t>band1_energy_ratio</t>
-  </si>
-  <si>
-    <t>AUC</t>
-  </si>
-  <si>
     <t>IQR</t>
   </si>
   <si>
+    <t>kurtosis</t>
+  </si>
+  <si>
+    <t>slope_min</t>
+  </si>
+  <si>
+    <t>slope_std</t>
+  </si>
+  <si>
+    <t>p90_p10_ratio</t>
+  </si>
+  <si>
+    <t>spectral_centroid</t>
+  </si>
+  <si>
+    <t>band2_energy_ratio</t>
+  </si>
+  <si>
+    <t>zero_crossing_rate</t>
+  </si>
+  <si>
+    <t>peak_max_height</t>
+  </si>
+  <si>
+    <t>peak_main_pos</t>
+  </si>
+  <si>
+    <t>signal_energy</t>
+  </si>
+  <si>
+    <t>CV</t>
+  </si>
+  <si>
     <t>slope_max</t>
   </si>
   <si>
-    <t>signal_energy</t>
-  </si>
-  <si>
-    <t>band2_energy_ratio</t>
-  </si>
-  <si>
-    <t>p90_p10_ratio</t>
-  </si>
-  <si>
-    <t>slope_min</t>
-  </si>
-  <si>
-    <t>spectral_centroid</t>
-  </si>
-  <si>
-    <t>slope_std</t>
-  </si>
-  <si>
-    <t>zero_crossing_rate</t>
-  </si>
-  <si>
-    <t>kurtosis</t>
-  </si>
-  <si>
-    <t>peak_max_height</t>
-  </si>
-  <si>
-    <t>peak_main_pos</t>
-  </si>
-  <si>
-    <t>CV</t>
+    <t>peak_max_width</t>
+  </si>
+  <si>
+    <t>peak_count</t>
+  </si>
+  <si>
+    <t>skewness</t>
   </si>
   <si>
     <t>first_high_pos</t>
   </si>
   <si>
+    <t>wavelet_cD1_std</t>
+  </si>
+  <si>
+    <t>range</t>
+  </si>
+  <si>
     <t>peak_mean_width</t>
   </si>
   <si>
+    <t>spectral_energy</t>
+  </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
     <t>band2_energy</t>
   </si>
   <si>
+    <t>peak_std_height</t>
+  </si>
+  <si>
+    <t>peak_last_pos</t>
+  </si>
+  <si>
+    <t>wavelet_cD3_std</t>
+  </si>
+  <si>
+    <t>std</t>
+  </si>
+  <si>
+    <t>signal_length</t>
+  </si>
+  <si>
+    <t>wavelet_cD2_std</t>
+  </si>
+  <si>
+    <t>wavelet_cD3_energy</t>
+  </si>
+  <si>
+    <t>fft_mag_max</t>
+  </si>
+  <si>
+    <t>band3_energy_ratio</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>dominant_freq</t>
+  </si>
+  <si>
     <t>valley_count</t>
-  </si>
-  <si>
-    <t>wavelet_cD1_std</t>
-  </si>
-  <si>
-    <t>peak_max_width</t>
-  </si>
-  <si>
-    <t>range</t>
-  </si>
-  <si>
-    <t>wavelet_cD2_std</t>
-  </si>
-  <si>
-    <t>std</t>
-  </si>
-  <si>
-    <t>dominant_freq</t>
-  </si>
-  <si>
-    <t>min</t>
-  </si>
-  <si>
-    <t>band3_energy_ratio</t>
-  </si>
-  <si>
-    <t>skewness</t>
-  </si>
-  <si>
-    <t>fft_mag_max</t>
-  </si>
-  <si>
-    <t>peak_last_pos</t>
-  </si>
-  <si>
-    <t>signal_length</t>
-  </si>
-  <si>
-    <t>wavelet_cD3_std</t>
-  </si>
-  <si>
-    <t>peak_count</t>
-  </si>
-  <si>
-    <t>spectral_energy</t>
-  </si>
-  <si>
-    <t>wavelet_cD3_energy</t>
-  </si>
-  <si>
-    <t>peak_std_height</t>
-  </si>
-  <si>
-    <t>mean</t>
   </si>
   <si>
     <t>peak_first_pos</t>
@@ -716,7 +716,7 @@
         <v>19</v>
       </c>
       <c r="C2">
-        <v>0.1591381192262276</v>
+        <v>0.1591381192262277</v>
       </c>
       <c r="D2" t="s">
         <v>9</v>
@@ -744,7 +744,7 @@
         <v>16</v>
       </c>
       <c r="C4">
-        <v>0.1119775820880677</v>
+        <v>0.1119775820880675</v>
       </c>
       <c r="D4" t="s">
         <v>24</v>
@@ -758,7 +758,7 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <v>0.0908590977204821</v>
+        <v>0.09085909772048202</v>
       </c>
       <c r="D5" t="s">
         <v>25</v>
@@ -786,7 +786,7 @@
         <v>38</v>
       </c>
       <c r="C7">
-        <v>-0.3020396303914649</v>
+        <v>-0.3020396303914751</v>
       </c>
       <c r="D7" t="s">
         <v>27</v>
@@ -800,7 +800,7 @@
         <v>38</v>
       </c>
       <c r="C8">
-        <v>-0.3020396303914706</v>
+        <v>-0.3020396303914754</v>
       </c>
       <c r="D8" t="s">
         <v>27</v>
@@ -814,7 +814,7 @@
         <v>38</v>
       </c>
       <c r="C9">
-        <v>-0.3020396303914799</v>
+        <v>-0.3020396303914761</v>
       </c>
       <c r="D9" t="s">
         <v>27</v>
@@ -873,13 +873,13 @@
         <v>1</v>
       </c>
       <c r="F2">
-        <v>0.00549865523086801</v>
+        <v>0.009821011648365463</v>
       </c>
       <c r="G2">
-        <v>0.1110782818648163</v>
+        <v>-0.02735564497726885</v>
       </c>
       <c r="H2">
-        <v>1.502158236852392E-09</v>
+        <v>0.1377612653534285</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -899,13 +899,13 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>0.009821011648365463</v>
+        <v>0.02523422267958875</v>
       </c>
       <c r="G3">
-        <v>-0.02735564497726885</v>
+        <v>0.2138175542021288</v>
       </c>
       <c r="H3">
-        <v>0.1377612653534285</v>
+        <v>8.487627874320932E-32</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -925,13 +925,13 @@
         <v>1</v>
       </c>
       <c r="F4">
-        <v>0.02523422267958875</v>
+        <v>0.00549865523086801</v>
       </c>
       <c r="G4">
-        <v>0.2138175542021288</v>
+        <v>0.1110782818648163</v>
       </c>
       <c r="H4">
-        <v>8.487627874320932E-32</v>
+        <v>1.502158236852392E-09</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -968,22 +968,22 @@
         <v>2</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6">
         <v>1</v>
       </c>
       <c r="F6">
-        <v>0.005146082862225398</v>
+        <v>0.05731493716539671</v>
       </c>
       <c r="G6">
-        <v>0.1202390767963869</v>
+        <v>0.2988528422305256</v>
       </c>
       <c r="H6">
-        <v>5.905596807141937E-11</v>
+        <v>7.984174917490527E-62</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1003,13 +1003,13 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>0.02072913454553404</v>
+        <v>0.03200907630035577</v>
       </c>
       <c r="G7">
-        <v>0.1986110102048823</v>
+        <v>-0.1094769033359784</v>
       </c>
       <c r="H7">
-        <v>1.401424378549223E-27</v>
+        <v>2.577521212571427E-09</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1020,22 +1020,22 @@
         <v>2</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
       <c r="F8">
-        <v>0.006548378834343893</v>
+        <v>0.01754307895227303</v>
       </c>
       <c r="G8">
-        <v>0.03104700235695857</v>
+        <v>0.1407052723387585</v>
       </c>
       <c r="H8">
-        <v>0.09207639231239179</v>
+        <v>1.710329654361346E-14</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1072,22 +1072,22 @@
         <v>2</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10">
         <v>1</v>
       </c>
       <c r="F10">
-        <v>0.03200907630035577</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>-0.1094769033359784</v>
+        <v>0.1123629329365884</v>
       </c>
       <c r="H10">
-        <v>2.577521212571427E-09</v>
+        <v>9.687342312506442E-10</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1098,22 +1098,22 @@
         <v>2</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11">
         <v>1</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>0.006548378834343893</v>
       </c>
       <c r="G11">
-        <v>0.1123629329365884</v>
+        <v>0.03104700235695857</v>
       </c>
       <c r="H11">
-        <v>9.687342312506442E-10</v>
+        <v>0.09207639231239179</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1124,22 +1124,22 @@
         <v>2</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12">
         <v>1</v>
       </c>
       <c r="F12">
-        <v>0.01754307895227303</v>
+        <v>0.07417534806562287</v>
       </c>
       <c r="G12">
-        <v>0.1407052723387585</v>
+        <v>0.2464811247000367</v>
       </c>
       <c r="H12">
-        <v>1.710329654361346E-14</v>
+        <v>5.236140342310394E-42</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1159,13 +1159,13 @@
         <v>1</v>
       </c>
       <c r="F13">
-        <v>0.07417534806562287</v>
+        <v>0.01768547067964743</v>
       </c>
       <c r="G13">
-        <v>0.2464811247000367</v>
+        <v>0.1711583551586446</v>
       </c>
       <c r="H13">
-        <v>5.236140342310394E-42</v>
+        <v>8.475132172070813E-21</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1185,13 +1185,13 @@
         <v>1</v>
       </c>
       <c r="F14">
-        <v>0.05731493716539671</v>
+        <v>0.03723789085394902</v>
       </c>
       <c r="G14">
-        <v>0.2988528422305256</v>
+        <v>0.1186944933835865</v>
       </c>
       <c r="H14">
-        <v>7.984174917490527E-62</v>
+        <v>1.037294292018274E-10</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1211,13 +1211,13 @@
         <v>1</v>
       </c>
       <c r="F15">
-        <v>0.01768547067964743</v>
+        <v>0.02072913454553404</v>
       </c>
       <c r="G15">
-        <v>0.1711583551586446</v>
+        <v>0.1986110102048823</v>
       </c>
       <c r="H15">
-        <v>8.475132172070813E-21</v>
+        <v>1.401424378549223E-27</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1237,13 +1237,13 @@
         <v>1</v>
       </c>
       <c r="F16">
-        <v>0.03723789085394902</v>
+        <v>0.01886985651344375</v>
       </c>
       <c r="G16">
-        <v>0.1186944933835865</v>
+        <v>-0.2658334978408707</v>
       </c>
       <c r="H16">
-        <v>1.037294292018274E-10</v>
+        <v>8.032049610475364E-49</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1254,22 +1254,22 @@
         <v>2</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="F17">
-        <v>0.01886985651344375</v>
+        <v>0.005146082862225398</v>
       </c>
       <c r="G17">
-        <v>-0.2658334978408707</v>
+        <v>0.1202390767963869</v>
       </c>
       <c r="H17">
-        <v>8.032049610475364E-49</v>
+        <v>5.905596807141937E-11</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1289,13 +1289,13 @@
         <v>1</v>
       </c>
       <c r="F18">
-        <v>0.0438628554196443</v>
+        <v>0.02070750587626691</v>
       </c>
       <c r="G18">
-        <v>0.0574221212752349</v>
+        <v>0.2048449701781561</v>
       </c>
       <c r="H18">
-        <v>0.001824385381363412</v>
+        <v>2.869676118301166E-29</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1315,13 +1315,13 @@
         <v>1</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>0.03516950609663283</v>
       </c>
       <c r="G19">
-        <v>0.1047294941308449</v>
+        <v>0.09199851623961416</v>
       </c>
       <c r="H19">
-        <v>1.221460257617864E-08</v>
+        <v>5.701862783338392E-07</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1341,13 +1341,13 @@
         <v>1</v>
       </c>
       <c r="F20">
-        <v>0.01164391449640689</v>
+        <v>0.02951097392287583</v>
       </c>
       <c r="G20">
-        <v>-0.03114698302244653</v>
+        <v>-0.1878262702326164</v>
       </c>
       <c r="H20">
-        <v>0.09103324268483054</v>
+        <v>8.652692818266743E-25</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1367,13 +1367,13 @@
         <v>1</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>0.0438628554196443</v>
       </c>
       <c r="G21">
-        <v>0.1355926075301449</v>
+        <v>0.0574221212752349</v>
       </c>
       <c r="H21">
-        <v>1.475540118603624E-13</v>
+        <v>0.001824385381363412</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1419,13 +1419,13 @@
         <v>1</v>
       </c>
       <c r="F23">
-        <v>0.02070750587626691</v>
+        <v>0.01051638257766463</v>
       </c>
       <c r="G23">
-        <v>0.2048449701781561</v>
+        <v>-0.01369191009713748</v>
       </c>
       <c r="H23">
-        <v>2.869676118301166E-29</v>
+        <v>0.4576330794546036</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1445,13 +1445,13 @@
         <v>1</v>
       </c>
       <c r="F24">
-        <v>0.01051638257766463</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>-0.01369191009713748</v>
+        <v>0.1047294941308449</v>
       </c>
       <c r="H24">
-        <v>0.4576330794546036</v>
+        <v>1.221460257617864E-08</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1471,13 +1471,13 @@
         <v>1</v>
       </c>
       <c r="F25">
-        <v>0.01515017913529437</v>
+        <v>0.007756576456852571</v>
       </c>
       <c r="G25">
-        <v>0.09540048027632948</v>
+        <v>-0.04548976647749594</v>
       </c>
       <c r="H25">
-        <v>2.13921132611932E-07</v>
+        <v>0.01355434683646457</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1497,13 +1497,13 @@
         <v>1</v>
       </c>
       <c r="F26">
-        <v>0.002942831275503544</v>
+        <v>0.03538293595809527</v>
       </c>
       <c r="G26">
-        <v>-0.08524723671707583</v>
+        <v>0.1846240973156884</v>
       </c>
       <c r="H26">
-        <v>3.610053665415079E-06</v>
+        <v>5.420556736330416E-24</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1523,13 +1523,13 @@
         <v>1</v>
       </c>
       <c r="F27">
-        <v>0.07434847645247622</v>
+        <v>0.01164391449640689</v>
       </c>
       <c r="G27">
-        <v>0.07824440845737834</v>
+        <v>-0.03114698302244653</v>
       </c>
       <c r="H27">
-        <v>2.129402957413155E-05</v>
+        <v>0.09103324268483054</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1549,13 +1549,13 @@
         <v>1</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>0.009667239864916688</v>
       </c>
       <c r="G28">
-        <v>0.2296195273811377</v>
+        <v>-0.05746636098243459</v>
       </c>
       <c r="H28">
-        <v>1.542938301579694E-36</v>
+        <v>0.001809551687529224</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1575,13 +1575,13 @@
         <v>1</v>
       </c>
       <c r="F29">
-        <v>0.001434970735492591</v>
+        <v>0.04692488271879736</v>
       </c>
       <c r="G29">
-        <v>0.02240877260712627</v>
+        <v>-0.02523558645428797</v>
       </c>
       <c r="H29">
-        <v>0.2240945035234869</v>
+        <v>0.1709624672148451</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1601,13 +1601,13 @@
         <v>1</v>
       </c>
       <c r="F30">
-        <v>0.02951097392287583</v>
+        <v>0.01264986478237962</v>
       </c>
       <c r="G30">
-        <v>-0.1878262702326164</v>
+        <v>0.06399692886502732</v>
       </c>
       <c r="H30">
-        <v>8.652692818266743E-25</v>
+        <v>0.0005107312877739539</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1627,13 +1627,13 @@
         <v>1</v>
       </c>
       <c r="F31">
-        <v>0.0002073033895264587</v>
+        <v>0.002942831275503544</v>
       </c>
       <c r="G31">
-        <v>-0.1117819402806436</v>
+        <v>-0.08524723671707583</v>
       </c>
       <c r="H31">
-        <v>1.182033348291729E-09</v>
+        <v>3.610053665415079E-06</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -1653,13 +1653,13 @@
         <v>1</v>
       </c>
       <c r="F32">
-        <v>0.04692488271879736</v>
+        <v>0.06242275155901567</v>
       </c>
       <c r="G32">
-        <v>-0.02523558645428797</v>
+        <v>0.2081474388615573</v>
       </c>
       <c r="H32">
-        <v>0.1709624672148451</v>
+        <v>3.471786326773779E-30</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1679,13 +1679,13 @@
         <v>1</v>
       </c>
       <c r="F33">
-        <v>0.06242275155901567</v>
+        <v>0.01515017913529437</v>
       </c>
       <c r="G33">
-        <v>0.2081474388615573</v>
+        <v>0.09540048027632948</v>
       </c>
       <c r="H33">
-        <v>3.471786326773779E-30</v>
+        <v>2.13921132611932E-07</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -1705,13 +1705,13 @@
         <v>1</v>
       </c>
       <c r="F34">
-        <v>0.01264986478237962</v>
+        <v>0.01662794639266618</v>
       </c>
       <c r="G34">
-        <v>0.06399692886502732</v>
+        <v>0.08144081073907809</v>
       </c>
       <c r="H34">
-        <v>0.0005107312877739539</v>
+        <v>9.64004287173663E-06</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -1731,13 +1731,13 @@
         <v>1</v>
       </c>
       <c r="F35">
-        <v>0.03516950609663283</v>
+        <v>0.0002073033895264587</v>
       </c>
       <c r="G35">
-        <v>0.09199851623961416</v>
+        <v>-0.1117819402806436</v>
       </c>
       <c r="H35">
-        <v>5.701862783338392E-07</v>
+        <v>1.182033348291729E-09</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -1757,13 +1757,13 @@
         <v>1</v>
       </c>
       <c r="F36">
-        <v>0.007756576456852571</v>
+        <v>0.001434970735492591</v>
       </c>
       <c r="G36">
-        <v>-0.04548976647749594</v>
+        <v>0.02240877260712627</v>
       </c>
       <c r="H36">
-        <v>0.01355434683646457</v>
+        <v>0.2240945035234869</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -1783,13 +1783,13 @@
         <v>1</v>
       </c>
       <c r="F37">
-        <v>0.01662794639266618</v>
+        <v>0</v>
       </c>
       <c r="G37">
-        <v>0.08144081073907809</v>
+        <v>0.2296195273811377</v>
       </c>
       <c r="H37">
-        <v>9.64004287173663E-06</v>
+        <v>1.542938301579694E-36</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -1809,13 +1809,13 @@
         <v>1</v>
       </c>
       <c r="F38">
-        <v>0.009667239864916688</v>
+        <v>0.07434847645247622</v>
       </c>
       <c r="G38">
-        <v>-0.05746636098243459</v>
+        <v>0.07824440845737834</v>
       </c>
       <c r="H38">
-        <v>0.001809551687529224</v>
+        <v>2.129402957413155E-05</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -1835,13 +1835,13 @@
         <v>1</v>
       </c>
       <c r="F39">
-        <v>0.03538293595809527</v>
+        <v>0</v>
       </c>
       <c r="G39">
-        <v>0.1846240973156884</v>
+        <v>0.1355926075301449</v>
       </c>
       <c r="H39">
-        <v>5.420556736330416E-24</v>
+        <v>1.475540118603624E-13</v>
       </c>
     </row>
   </sheetData>
@@ -1870,7 +1870,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="B2">
         <v>0.07434847645247622</v>
@@ -1884,7 +1884,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B3">
         <v>0.07417534806562287</v>
@@ -1898,7 +1898,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B4">
         <v>0.06242275155901567</v>
@@ -1912,7 +1912,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>0.05731493716539671</v>
@@ -1926,7 +1926,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B6">
         <v>0.04692488271879736</v>
@@ -1954,7 +1954,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B8">
         <v>0.0438628554196443</v>
@@ -1968,7 +1968,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B9">
         <v>0.03723789085394902</v>
@@ -1982,7 +1982,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B10">
         <v>0.03538293595809527</v>
@@ -1996,7 +1996,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="B11">
         <v>0.03516950609663283</v>
@@ -2010,7 +2010,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B12">
         <v>0.03200907630035577</v>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="B13">
         <v>0.02951097392287583</v>
@@ -2038,7 +2038,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B14">
         <v>0.02523422267958875</v>
@@ -2052,7 +2052,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="B15">
         <v>0.02072913454553404</v>
@@ -2066,7 +2066,7 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B16">
         <v>0.02070750587626691</v>
@@ -2080,7 +2080,7 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B17">
         <v>0.01886985651344375</v>
@@ -2094,7 +2094,7 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B18">
         <v>0.01768547067964743</v>
@@ -2108,7 +2108,7 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B19">
         <v>0.01754307895227303</v>
@@ -2122,7 +2122,7 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B20">
         <v>0.01662794639266618</v>
@@ -2136,7 +2136,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B21">
         <v>0.01515017913529437</v>
@@ -2164,7 +2164,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B23">
         <v>0.01264986478237962</v>
@@ -2178,7 +2178,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B24">
         <v>0.01164391449640689</v>
@@ -2192,7 +2192,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B25">
         <v>0.01051638257766463</v>
@@ -2206,7 +2206,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B26">
         <v>0.009821011648365463</v>
@@ -2220,7 +2220,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B27">
         <v>0.009667239864916688</v>
@@ -2234,7 +2234,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B28">
         <v>0.007756576456852571</v>
@@ -2248,7 +2248,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B29">
         <v>0.006548378834343893</v>
@@ -2262,7 +2262,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B30">
         <v>0.00549865523086801</v>
@@ -2276,7 +2276,7 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="B31">
         <v>0.005146082862225398</v>
@@ -2290,7 +2290,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B32">
         <v>0.002942831275503544</v>
@@ -2318,7 +2318,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B34">
         <v>0.001434970735492591</v>
@@ -2332,7 +2332,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B35">
         <v>0.0002073033895264587</v>
@@ -2346,7 +2346,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="B36">
         <v>0</v>
@@ -2360,7 +2360,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -2388,7 +2388,7 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -2416,7 +2416,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -2476,7 +2476,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B2">
         <v>1475.943670683168</v>
@@ -2484,7 +2484,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="B3">
         <v>434.7492937335367</v>
@@ -2492,7 +2492,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B4">
         <v>413.7444661243916</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5">
         <v>404.7850590942015</v>
@@ -2508,7 +2508,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B6">
         <v>359.6857379269365</v>
@@ -2516,7 +2516,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7">
         <v>291.1168450538412</v>
@@ -2524,7 +2524,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B8">
         <v>242.6144523334943</v>
@@ -2540,7 +2540,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10">
         <v>194.5523729317617</v>
@@ -2548,7 +2548,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B11">
         <v>129.2392535271388</v>
@@ -2556,7 +2556,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12">
         <v>120.5772091217362</v>
@@ -2564,7 +2564,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B13">
         <v>105.6837534342637</v>
@@ -2572,7 +2572,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B14">
         <v>93.02101771977938</v>
@@ -2596,7 +2596,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="B17">
         <v>63.27955130643879</v>
@@ -2612,7 +2612,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B19">
         <v>51.15479374765392</v>
@@ -2620,7 +2620,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B20">
         <v>37.33028582860905</v>
@@ -2628,7 +2628,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B21">
         <v>35.99255555858554</v>
@@ -2636,7 +2636,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="B22">
         <v>35.35808744079256</v>
@@ -2644,7 +2644,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="B23">
         <v>31.18565164428958</v>
@@ -2652,7 +2652,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B24">
         <v>28.00914104991081</v>
@@ -2668,7 +2668,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B26">
         <v>22.41419271978275</v>
@@ -2676,7 +2676,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B27">
         <v>21.32480698376821</v>
@@ -2684,7 +2684,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B28">
         <v>20.88415948798974</v>
@@ -2692,7 +2692,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="B29">
         <v>19.12110947388943</v>
@@ -2700,7 +2700,7 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B30">
         <v>18.67727752188462</v>
@@ -2716,7 +2716,7 @@
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B32">
         <v>18.36537712412012</v>
@@ -2724,7 +2724,7 @@
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B33">
         <v>14.48594287431152</v>
@@ -2732,7 +2732,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B34">
         <v>12.87694577773936</v>
@@ -2740,7 +2740,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B35">
         <v>11.73411018848921</v>
@@ -2748,7 +2748,7 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B36">
         <v>11.63861143778816</v>
@@ -2764,7 +2764,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B38">
         <v>10.66653606524847</v>
@@ -2772,7 +2772,7 @@
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="B39">
         <v>7.968052388644953</v>
@@ -2780,7 +2780,7 @@
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B40">
         <v>7.00616397049654</v>
@@ -2788,7 +2788,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B41">
         <v>6.118056739187805</v>
@@ -2796,7 +2796,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B42">
         <v>4.74652599951668</v>
@@ -2804,7 +2804,7 @@
     </row>
     <row r="43" spans="1:2">
       <c r="A43" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B43">
         <v>3.690056290732489</v>
@@ -2833,7 +2833,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B2">
         <v>244.1920131508512</v>
@@ -2844,7 +2844,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B3">
         <v>214.142067733607</v>
@@ -2855,7 +2855,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4">
         <v>148.8642549036453</v>
@@ -2877,7 +2877,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>33.07620137307747</v>
@@ -2888,7 +2888,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B7">
         <v>31.74208716959095</v>
@@ -2899,7 +2899,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B8">
         <v>31.60672691275246</v>
@@ -2910,7 +2910,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="B9">
         <v>24.88660907087396</v>
@@ -2921,7 +2921,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B10">
         <v>22.25432808888731</v>
@@ -2932,7 +2932,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B11">
         <v>16.65742391636174</v>
@@ -2943,7 +2943,7 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B12">
         <v>15.86982844026153</v>
@@ -2965,7 +2965,7 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B14">
         <v>7.476063836633235</v>
@@ -2976,7 +2976,7 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B15">
         <v>6.854743279622218</v>
@@ -2987,7 +2987,7 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B16">
         <v>6.285738475955339</v>
@@ -2998,7 +2998,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B17">
         <v>5.365975364875827</v>
@@ -3009,7 +3009,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B18">
         <v>5.262060465534107</v>
@@ -3020,7 +3020,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B19">
         <v>5.098843475181286</v>
@@ -3031,7 +3031,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B20">
         <v>5.082278982581335</v>
@@ -3042,7 +3042,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B21">
         <v>146.0462147113818</v>
@@ -3064,7 +3064,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23">
         <v>33.05594027348305</v>
@@ -3075,7 +3075,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B24">
         <v>31.40629671376154</v>
@@ -3086,7 +3086,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B25">
         <v>25.39763719197679</v>
@@ -3097,7 +3097,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="B26">
         <v>24.23710466230549</v>
@@ -3108,7 +3108,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B27">
         <v>22.51073730600591</v>
@@ -3119,7 +3119,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B28">
         <v>21.86123963729892</v>
@@ -3130,7 +3130,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B29">
         <v>16.65741955902392</v>
@@ -3141,7 +3141,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B30">
         <v>14.6786092067813</v>
@@ -3163,7 +3163,7 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B32">
         <v>7.474639549836925</v>
@@ -3174,7 +3174,7 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B33">
         <v>6.291375912561315</v>
@@ -3185,7 +3185,7 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B34">
         <v>5.199980386062538</v>
@@ -3196,7 +3196,7 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B35">
         <v>5.082277296348062</v>
@@ -3207,7 +3207,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B36">
         <v>5.075812036103986</v>
@@ -3218,7 +3218,7 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B37">
         <v>4.932398890841717</v>
@@ -3229,7 +3229,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B38">
         <v>3.889796808693125</v>
@@ -3240,7 +3240,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B39">
         <v>29.91119580117911</v>
@@ -3251,7 +3251,7 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B40">
         <v>29.59419050370359</v>
@@ -3262,7 +3262,7 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="B41">
         <v>23.91783631726542</v>
@@ -3284,7 +3284,7 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B43">
         <v>21.67470880704602</v>
@@ -3295,7 +3295,7 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B44">
         <v>21.48395163842845</v>
@@ -3306,7 +3306,7 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B45">
         <v>14.42809518047245</v>
@@ -3317,7 +3317,7 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B46">
         <v>13.61733886429231</v>
@@ -3328,7 +3328,7 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B47">
         <v>13.45105164643281</v>
@@ -3350,7 +3350,7 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B49">
         <v>6.912002452693454</v>
@@ -3361,7 +3361,7 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B50">
         <v>6.012371620899786</v>
@@ -3372,7 +3372,7 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B51">
         <v>5.199721684760331</v>
@@ -3383,7 +3383,7 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B52">
         <v>5.080093556522899</v>
@@ -3394,7 +3394,7 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B53">
         <v>5.009640078879248</v>
@@ -3405,7 +3405,7 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B54">
         <v>4.93134079698581</v>
@@ -3416,7 +3416,7 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B55">
         <v>3.855159801030515</v>
@@ -3427,7 +3427,7 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B56">
         <v>25.38791968038181</v>
@@ -3438,7 +3438,7 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="B57">
         <v>23.85641516276298</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B58">
         <v>21.61463226598549</v>
@@ -3460,7 +3460,7 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B59">
         <v>21.48322667342385</v>
@@ -3482,7 +3482,7 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B61">
         <v>14.42775130647092</v>
@@ -3493,7 +3493,7 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B62">
         <v>13.45809231271252</v>
@@ -3504,7 +3504,7 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B63">
         <v>12.782101842674</v>
@@ -3526,7 +3526,7 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B65">
         <v>5.737728269904268</v>
@@ -3537,7 +3537,7 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B66">
         <v>5.075015939063271</v>
@@ -3548,7 +3548,7 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B67">
         <v>4.892260777931048</v>
@@ -3559,7 +3559,7 @@
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B68">
         <v>4.883896218065412</v>
@@ -3570,7 +3570,7 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B69">
         <v>4.448225066012912</v>
@@ -3581,7 +3581,7 @@
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B70">
         <v>3.854942100429904</v>
@@ -3592,7 +3592,7 @@
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B71">
         <v>2.459502659885041</v>
@@ -3603,7 +3603,7 @@
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="B72">
         <v>23.85623781472384</v>
@@ -3614,7 +3614,7 @@
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B73">
         <v>21.6146203966318</v>
@@ -3625,7 +3625,7 @@
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B74">
         <v>18.81481920565012</v>
@@ -3647,7 +3647,7 @@
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B76">
         <v>13.91024909058624</v>
@@ -3658,7 +3658,7 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B77">
         <v>12.45557985262191</v>
@@ -3669,7 +3669,7 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B78">
         <v>11.09140340761202</v>
@@ -3691,7 +3691,7 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B80">
         <v>5.171515216873476</v>
@@ -3702,7 +3702,7 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B81">
         <v>5.046335738450336</v>
@@ -3713,7 +3713,7 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B82">
         <v>4.84912659517585</v>
@@ -3724,7 +3724,7 @@
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B83">
         <v>4.12523699824097</v>
@@ -3735,7 +3735,7 @@
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B84">
         <v>3.264778674149973</v>
@@ -3746,7 +3746,7 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B85">
         <v>2.345004512841142</v>
@@ -3757,7 +3757,7 @@
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B86">
         <v>2.188887471648316</v>
@@ -3768,7 +3768,7 @@
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B87">
         <v>17.96713872664587</v>
@@ -3790,7 +3790,7 @@
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B89">
         <v>13.90785809293445</v>
@@ -3801,7 +3801,7 @@
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B90">
         <v>12.28042807192004</v>
@@ -3812,7 +3812,7 @@
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B91">
         <v>11.02596815767474</v>
@@ -3834,7 +3834,7 @@
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B93">
         <v>5.307425658989214</v>
@@ -3845,7 +3845,7 @@
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B94">
         <v>5.15696262309422</v>
@@ -3856,7 +3856,7 @@
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B95">
         <v>5.025958223617559</v>
@@ -3867,7 +3867,7 @@
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B96">
         <v>4.559540086075645</v>
@@ -3878,7 +3878,7 @@
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B97">
         <v>4.088512629498615</v>
@@ -3889,7 +3889,7 @@
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B98">
         <v>3.262480452851506</v>
@@ -3900,7 +3900,7 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B99">
         <v>2.344583628123123</v>
@@ -3911,7 +3911,7 @@
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B100">
         <v>2.181834906302042</v>
@@ -3922,7 +3922,7 @@
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B101">
         <v>13.75341983266999</v>
@@ -3944,7 +3944,7 @@
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B103">
         <v>11.06138258872647</v>
@@ -3955,7 +3955,7 @@
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B104">
         <v>10.833772538098</v>
@@ -3977,7 +3977,7 @@
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B106">
         <v>5.150459181951671</v>
@@ -3988,7 +3988,7 @@
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B107">
         <v>4.962146239113817</v>
@@ -3999,7 +3999,7 @@
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B108">
         <v>4.736189620900321</v>
@@ -4010,7 +4010,7 @@
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B109">
         <v>4.041371245337825</v>
@@ -4021,7 +4021,7 @@
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B110">
         <v>3.810333695077866</v>
@@ -4032,7 +4032,7 @@
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B111">
         <v>2.469146714571565</v>
@@ -4043,7 +4043,7 @@
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B112">
         <v>2.315666720483321</v>
@@ -4054,7 +4054,7 @@
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B113">
         <v>1.845736804895733</v>
@@ -4076,7 +4076,7 @@
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B115">
         <v>11.02682097480001</v>
@@ -4087,7 +4087,7 @@
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B116">
         <v>10.71726346162865</v>
@@ -4109,7 +4109,7 @@
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B118">
         <v>4.541491104339819</v>
@@ -4120,7 +4120,7 @@
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B119">
         <v>4.40199055534352</v>
@@ -4131,7 +4131,7 @@
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B120">
         <v>3.998448528416785</v>
@@ -4142,7 +4142,7 @@
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B121">
         <v>3.756684000068823</v>
@@ -4153,7 +4153,7 @@
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B122">
         <v>3.626449031258577</v>
@@ -4164,7 +4164,7 @@
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B123">
         <v>2.450760100415931</v>
@@ -4175,7 +4175,7 @@
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B124">
         <v>2.307618156346136</v>
@@ -4186,7 +4186,7 @@
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B125">
         <v>1.802873101064548</v>
@@ -4197,7 +4197,7 @@
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B126">
         <v>10.70402242239174</v>
@@ -4208,7 +4208,7 @@
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B127">
         <v>6.898702948229213</v>
@@ -4230,7 +4230,7 @@
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B129">
         <v>4.54131082867941</v>
@@ -4241,7 +4241,7 @@
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B130">
         <v>3.93368209894374</v>
@@ -4252,7 +4252,7 @@
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B131">
         <v>3.730055752457127</v>
@@ -4263,7 +4263,7 @@
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B132">
         <v>3.719819445043717</v>
@@ -4274,7 +4274,7 @@
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B133">
         <v>3.597872454305945</v>
@@ -4285,7 +4285,7 @@
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B134">
         <v>2.303277618676784</v>
@@ -4296,7 +4296,7 @@
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B135">
         <v>2.192392765463522</v>
@@ -4307,7 +4307,7 @@
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B136">
         <v>1.798183117779326</v>
@@ -4336,7 +4336,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B2">
         <v>10.70402242239174</v>
@@ -4344,7 +4344,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B3">
         <v>6.898702948229213</v>
@@ -4360,7 +4360,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B5">
         <v>4.54131082867941</v>
@@ -4368,7 +4368,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6">
         <v>3.93368209894374</v>
@@ -4376,7 +4376,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B7">
         <v>3.730055752457127</v>
@@ -4384,7 +4384,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B8">
         <v>3.719819445043717</v>
@@ -4392,7 +4392,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B9">
         <v>3.597872454305945</v>
@@ -4400,7 +4400,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B10">
         <v>2.303277618676784</v>
@@ -4408,7 +4408,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B11">
         <v>2.192392765463522</v>
@@ -4416,7 +4416,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="B12">
         <v>1.798183117779326</v>
@@ -4439,42 +4439,42 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:1">
@@ -4484,12 +4484,12 @@
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>